<commit_message>
specs : onglet Aventures dans cartes.xlsx (brouillon Asteroides/Trois lunes/Police)
Transcrit tel quel le contenu fourni par l'utilisateur (nom/description/3 choix par
aventure), avec une colonne Notes signalant les mecaniques manquantes cote moteur pour
chaque choix. Pas encore reporte dans specs.md ni implemente (specs.md 2.4 etape 7).
</commit_message>
<xml_diff>
--- a/specs/cartes.xlsx
+++ b/specs/cartes.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Legende" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cartes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Aventures" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cartes'!$A$1:$L$45</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,21 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -87,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,6 +117,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2674,4 +2698,222 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Registre des aventures - Space Fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Brouillon issu des aventures decrites par l'utilisateur (cf. specs.md 2.4 etape 7, contenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>encore a specifier completement - pas encore reporte dans specs.md ni implemente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Colonne Image : fond dedie dans assets/aventure/ (sauvegardes, pas encore branches au code).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Choix 1/2/3 : effet du choix en langage naturel, tel que fourni - pas encore traduit en</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>mecanique de moteur (contrairement a Cartes, aucune colonne Jouable/Effet ici pour l'instant).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Miroir humainement modifiable, comme Cartes - pas relu par le code. Voir CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Choix 1</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Choix 2</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Choix 3</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Asteroides</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>assets/aventure/champ_asteroides.png</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Poursuivi par des pirates de l'espace, vous n'avez plus le choix : vaincre ou perir ! A moins que...</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Traverser le champ d'asteroides - perdez 5 PV sur un de vos modules.
+PUIS ces asteroides n'en finissent plus, perdez encore 5 PV.
+PUIS tout pres de la sortie, vous reperez des debris que vous recuperez (tirer une carte au hasard et la proposer gratuitement au joueur : il la prend ou il passe).</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Affronter les pirates (lance un combat aleatoire contre 3 ennemis Small).</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Choix 1 : reutilise le tirage de carte gratuit (nouveau : hors flux de recompense standard, carte non ajoutee au deck si le joueur passe). Choix 2 : reutilise creer_flotte, mais avec un nombre/une taille d'ennemis fixes plutot que le tirage habituel lie au niveau (specs.md 2.3/10.3, deja approximatif). Choix 3 vide - a combler ou assumer un choix binaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Trois lunes</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>assets/aventure/trois_lunes.png</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Un havre de paix au milieu de la galaxie. Aucune forme de vie intelligente, des animaux de taille raisonnable, de l'eau, des fruits et des legumes sauvages partout. Il est temps de faire une pause.</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Reparer le vaisseau - chaque module regagne 5 PV.</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Ameliorer - un module gagne 10 PV max (meme montant qu'en Station service).</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Bricoler - retirer une carte du deck.</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Choix 1 : nouveau (reparer_module existant ne s'applique qu'a UN module choisi, ici tous les modules a la fois, montant different : 5 au lieu de PV_REPARATION=20). Choix 2 : reutilise ameliorer_module (PV_AMELIORATION=10) sur un module au choix. Choix 3 : nouveau (aucune fonction de retrait de carte cote gameplay actuellement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Police</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>assets/aventure/police.png</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Pas de bol, votre dernier achat n'est pas aux normes. Et la police de l'espace ne plaisante pas trop dans le coin...</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Confiscation - supprimer la carte &lt;carte tiree au sort du deck&gt; de votre deck.</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Mettre aux normes - payez &lt;la moitie du cout de la carte en magasin&gt;.</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Detourner l'attention - changer la carte (une seule fois).</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Suppose une carte deja tiree au sort avant meme l'affichage des choix (le texte des choix 1/2 la reference). Choix 2 : "cout de la carte en magasin" suppose la Planete commerciale (prix par carte pas encore definis, specs.md 9.1). Choix 3 : "changer la carte" ambigu - retirer cette carte sans autre effet ? La remplacer par une autre tiree au hasard ? A clarifier.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs : tranche les points ouverts des 3 premieres aventures (specs.md 2.5)
Decisions prises avec l'utilisateur : Asteroides en un seul ecran sequence (pas de
moteur narratif generique), combat approxime a 3 ennemis du pool actuel (pas de taille
S/M/L pour l'instant), cout de "Mettre aux normes" (Police) remplace par un montant fixe
de 10 Argent (invente, la Planete commerciale n'ayant pas de prix par carte), "Detourner
l'attention" limite a une fois par Aventure (pas par run, rien a persister sur Partie).

Report dans specs.md (nouvelle section 2.5) et dans l'onglet Aventures de cartes.xlsx.
Aucun code touche - toujours pas implemente, l'etape Aventure utilise encore l'ecran
generique EcranEtapePlaceholder.
</commit_message>
<xml_diff>
--- a/specs/cartes.xlsx
+++ b/specs/cartes.xlsx
@@ -2725,6 +2725,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2739,6 +2740,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
@@ -2760,6 +2762,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -2767,6 +2770,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
@@ -2835,7 +2839,7 @@
       <c r="F13" s="10" t="inlineStr"/>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Choix 1 : reutilise le tirage de carte gratuit (nouveau : hors flux de recompense standard, carte non ajoutee au deck si le joueur passe). Choix 2 : reutilise creer_flotte, mais avec un nombre/une taille d'ennemis fixes plutot que le tirage habituel lie au niveau (specs.md 2.3/10.3, deja approximatif). Choix 3 vide - a combler ou assumer un choix binaire.</t>
+          <t>Decisions prises (voir specs.md 2.5) : sequence en 3 temps sur UN SEUL ecran (bouton Continuer entre chaque etape, pas de fenetres separees) ; module touche par les -5 PV choisi par un clic du joueur ; combat = approximation "3 ennemis tires du pool actuel" (pas de taille S/M/L, absente de config/ennemis.json - implementer ce tag reste une piste ouverte, cf. specs.md 3.2/9.1/10.3, mais pas un prerequis pour cette Aventure). Choix 3 confirme vide (binaire assume).</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2876,7 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Choix 1 : nouveau (reparer_module existant ne s'applique qu'a UN module choisi, ici tous les modules a la fois, montant different : 5 au lieu de PV_REPARATION=20). Choix 2 : reutilise ameliorer_module (PV_AMELIORATION=10) sur un module au choix. Choix 3 : nouveau (aucune fonction de retrait de carte cote gameplay actuellement).</t>
+          <t>Decisions confirmees (specs.md 2.5) : Reparer = nouveau soin groupe (chaque module +5 PV, distinct de reparer_module qui ne cible qu'un module) ; Ameliorer = reutilise ameliorer_module tel quel sur le module clique ; Bricoler = nouvelle fonction de retrait de carte (aucune n'existe encore, seul ajouter_carte existe).</t>
         </is>
       </c>
     </row>
@@ -2899,17 +2903,17 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Mettre aux normes - payez &lt;la moitie du cout de la carte en magasin&gt;.</t>
+          <t>Mettre aux normes - payez 10 Argent (montant fixe, pas un pourcentage du prix en magasin).</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Detourner l'attention - changer la carte (une seule fois).</t>
+          <t>Detourner l'attention - tire une seconde carte au hasard qui remplace la premiere, revient a l'ecran avec seulement 2 choix restants (Confiscation/Mettre aux normes).</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Suppose une carte deja tiree au sort avant meme l'affichage des choix (le texte des choix 1/2 la reference). Choix 2 : "cout de la carte en magasin" suppose la Planete commerciale (prix par carte pas encore definis, specs.md 9.1). Choix 3 : "changer la carte" ambigu - retirer cette carte sans autre effet ? La remplacer par une autre tiree au hasard ? A clarifier.</t>
+          <t>Decisions prises (specs.md 2.5) : le prix "en magasin" de la carte n'existe pas encore (Planete commerciale non chiffree) -&gt; remplace par un montant fixe de 10 Argent, invente par symetrie avec les autres montants (a ajuster en playtest, meme statut que ARGENT_PAR_ENNEMI_TUE/COUT_ACTION_STATION_SERVICE). "Une seule fois" = une seule fois PAR AVENTURE (pas par run) : rien a persister sur Partie, purement local a l'ecran.</t>
         </is>
       </c>
     </row>

</xml_diff>